<commit_message>
Add points for cqsflhc7vaul90l2d4ipzzzmc_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/cqsflhc7vaul90l2d4ipzzzmc_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/cqsflhc7vaul90l2d4ipzzzmc_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG23"/>
+  <dimension ref="A1:BG28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="AD2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -955,14 +955,14 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
@@ -991,7 +991,7 @@
         </is>
       </c>
       <c r="AD3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -1008,21 +1008,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>0.67043016</v>
+        <v>0.7378233199999999</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>+0.23</t>
+          <t>+0.32</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1040,7 +1040,7 @@
         <v>4</v>
       </c>
       <c r="AS3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT3" t="n">
         <v>0</v>
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="BE3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="BF3" t="n">
         <v>1</v>
@@ -1142,14 +1142,14 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="S4" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
@@ -1178,7 +1178,7 @@
         </is>
       </c>
       <c r="AD4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
@@ -1195,77 +1195,77 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0.73217924</v>
+        <v>0.85672589</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>+0.30</t>
+          <t>+0.44</t>
         </is>
       </c>
       <c r="AK4" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>83</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="inlineStr">
+        <is>
+          <t>DEF</t>
+        </is>
+      </c>
+      <c r="BE4" t="n">
         <v>5</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>73</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AR4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS4" t="n">
-        <v>2</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD4" t="inlineStr">
-        <is>
-          <t>DEF</t>
-        </is>
-      </c>
-      <c r="BE4" t="n">
-        <v>3</v>
       </c>
       <c r="BF4" t="n">
         <v>2</v>
@@ -1329,14 +1329,14 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="S5" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="AD5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1382,30 +1382,30 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0.29498066</v>
+        <v>1.03525483</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>-0.14</t>
+          <t>+0.61</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN5" t="n">
         <v>0</v>
       </c>
       <c r="AO5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ5" t="n">
         <v>0</v>
@@ -1451,7 +1451,7 @@
         <v>0</v>
       </c>
       <c r="BF5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG5" t="n">
         <v>0</v>
@@ -1512,14 +1512,14 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1527,7 +1527,7 @@
         </is>
       </c>
       <c r="S6" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
@@ -1548,7 +1548,7 @@
         </is>
       </c>
       <c r="AD6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
@@ -1565,21 +1565,21 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.8177353000000001</v>
+        <v>0.79271537</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>+0.38</t>
+          <t>+0.37</t>
         </is>
       </c>
       <c r="AK6" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="AL6" t="n">
         <v>0</v>
       </c>
       <c r="AM6" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN6" t="n">
         <v>0</v>
@@ -1699,14 +1699,14 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -1714,7 +1714,7 @@
         </is>
       </c>
       <c r="S7" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
@@ -1735,7 +1735,7 @@
         </is>
       </c>
       <c r="AD7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE7" t="n">
         <v>0</v>
@@ -1752,21 +1752,21 @@
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0.46630535</v>
+        <v>0.46666035</v>
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>+0.03</t>
+          <t>+0.05</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
       </c>
       <c r="AM7" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN7" t="n">
         <v>0</v>
@@ -1886,7 +1886,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="U8" t="n">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="V8" t="inlineStr"/>
       <c r="W8" t="inlineStr"/>
@@ -1932,7 +1932,7 @@
         </is>
       </c>
       <c r="AD8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
@@ -1949,11 +1949,11 @@
         </is>
       </c>
       <c r="AI8" t="n">
-        <v>2.19269588</v>
+        <v>2.25889953</v>
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>+1.76</t>
+          <t>+1.84</t>
         </is>
       </c>
       <c r="AK8" t="n">
@@ -1963,7 +1963,7 @@
         <v>0</v>
       </c>
       <c r="AM8" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN8" t="n">
         <v>0</v>
@@ -2083,14 +2083,14 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="S9" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="AD9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE9" t="n">
         <v>0</v>
@@ -2136,21 +2136,21 @@
         </is>
       </c>
       <c r="AI9" t="n">
-        <v>0.14230376</v>
+        <v>0.19635666</v>
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>-0.29</t>
+          <t>-0.22</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
       </c>
       <c r="AM9" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN9" t="n">
         <v>0</v>
@@ -2165,16 +2165,16 @@
         <v>0</v>
       </c>
       <c r="AR9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AS9" t="n">
         <v>0</v>
       </c>
       <c r="AT9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV9" t="n">
         <v>0</v>
@@ -2206,7 +2206,7 @@
         </is>
       </c>
       <c r="BE9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="BF9" t="n">
         <v>0</v>
@@ -2270,14 +2270,14 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2285,7 +2285,7 @@
         </is>
       </c>
       <c r="S10" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
@@ -2306,7 +2306,7 @@
         </is>
       </c>
       <c r="AD10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE10" t="n">
         <v>0</v>
@@ -2323,11 +2323,11 @@
         </is>
       </c>
       <c r="AI10" t="n">
-        <v>1.2662073</v>
+        <v>1.28469531</v>
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>+0.83</t>
+          <t>+0.86</t>
         </is>
       </c>
       <c r="AK10" t="n">
@@ -2337,7 +2337,7 @@
         <v>0</v>
       </c>
       <c r="AM10" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN10" t="n">
         <v>1</v>
@@ -2349,10 +2349,10 @@
         <v>0</v>
       </c>
       <c r="AQ10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="AR10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AS10" t="n">
         <v>0</v>
@@ -2393,10 +2393,10 @@
         </is>
       </c>
       <c r="BE10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BF10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="BG10" t="n">
         <v>8</v>
@@ -2443,10 +2443,12 @@
           <t>ckaqxlw257qzj8vjdumvwbaad</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -2457,7 +2459,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -2468,7 +2470,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2484,7 +2486,7 @@
         </is>
       </c>
       <c r="U11" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
@@ -2512,7 +2514,7 @@
         <v>0.1</v>
       </c>
       <c r="AG11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -2520,21 +2522,21 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.35178459</v>
+        <v>0.38766864</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.03</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2549,7 +2551,7 @@
         <v>0</v>
       </c>
       <c r="AR11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS11" t="n">
         <v>0</v>
@@ -2590,7 +2592,7 @@
         </is>
       </c>
       <c r="BE11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="BF11" t="n">
         <v>0</v>
@@ -2654,14 +2656,18 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>73</v>
-      </c>
-      <c r="O12" t="inlineStr"/>
+        <v>83</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2669,10 +2675,16 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>73</v>
-      </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+        <v>79.40000000000001</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>3.6</v>
+      </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
@@ -2690,7 +2702,7 @@
         </is>
       </c>
       <c r="AD12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AE12" t="n">
         <v>0</v>
@@ -2707,11 +2719,11 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>0.88675785</v>
+        <v>1.15396199</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>+0.45</t>
+          <t>+0.73</t>
         </is>
       </c>
       <c r="AK12" t="n">
@@ -2721,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -2751,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="AW12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX12" t="n">
         <v>0</v>
@@ -2780,7 +2792,7 @@
         <v>6</v>
       </c>
       <c r="BF12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="BG12" t="n">
         <v>2</v>
@@ -2794,37 +2806,37 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>4pz87gsel7183b7kcadw1dwzv</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>É. Mendy</t>
+          <t>B. Barcola</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>16</t>
+          <t xml:space="preserve"> 12</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>22s7hpp9k5ihtc2pwiaytdp05</t>
+          <t>a71n80h977h7fu99ftnri5zsa</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -2833,33 +2845,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>79</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2</v>
+      </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N13" t="n">
-        <v>73</v>
-      </c>
-      <c r="O13" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="Q13" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="S13" t="n">
-        <v>73</v>
-      </c>
-      <c r="T13" t="inlineStr"/>
-      <c r="U13" t="inlineStr"/>
+        <v>0.4</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>3.6</v>
+      </c>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr"/>
@@ -2868,38 +2894,50 @@
       <c r="AA13" t="inlineStr"/>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>2wk1549tkz80oet8226euj7jp</t>
+          <t>4pz87gsel7183b7kcadw1dwzv</t>
         </is>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>France</t>
         </is>
       </c>
       <c r="AD13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF13" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>B. Barcola</t>
+        </is>
+      </c>
+      <c r="AI13" t="n">
+        <v>0.9656987899999999</v>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>+0.55</t>
+        </is>
+      </c>
+      <c r="AK13" t="n">
+        <v>5</v>
+      </c>
       <c r="AL13" t="n">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="AM13" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO13" t="n">
         <v>0</v>
@@ -2908,53 +2946,57 @@
         <v>0</v>
       </c>
       <c r="AQ13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
+      <c r="BE13" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF13" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG13" t="n">
         <v>5</v>
-      </c>
-      <c r="AS13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV13" t="n">
-        <v>3</v>
-      </c>
-      <c r="AW13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD13" t="inlineStr"/>
-      <c r="BE13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF13" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG13" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -2970,17 +3012,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>K. Diatta</t>
+          <t>É. Mendy</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 15</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -2990,12 +3032,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>f5j3vhj805xtkos7l538u0d7t</t>
+          <t>22s7hpp9k5ihtc2pwiaytdp05</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -3012,22 +3054,22 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
@@ -3051,35 +3093,23 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF14" t="n">
-        <v>-0.2</v>
+        <v>0</v>
       </c>
       <c r="AG14" t="n">
         <v>1</v>
       </c>
-      <c r="AH14" t="inlineStr">
-        <is>
-          <t>K. Diatta</t>
-        </is>
-      </c>
-      <c r="AI14" t="n">
-        <v>0.2705196599999999</v>
-      </c>
-      <c r="AJ14" t="inlineStr">
-        <is>
-          <t>-0.17</t>
-        </is>
-      </c>
-      <c r="AK14" t="n">
-        <v>13</v>
-      </c>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
       <c r="AL14" t="n">
         <v>0</v>
       </c>
       <c r="AM14" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3091,22 +3121,22 @@
         <v>0</v>
       </c>
       <c r="AQ14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AR14" t="n">
+        <v>5</v>
+      </c>
+      <c r="AS14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV14" t="n">
         <v>4</v>
-      </c>
-      <c r="AS14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AU14" t="n">
-        <v>4</v>
-      </c>
-      <c r="AV14" t="n">
-        <v>0</v>
       </c>
       <c r="AW14" t="n">
         <v>0</v>
@@ -3134,7 +3164,7 @@
         <v>0</v>
       </c>
       <c r="BF14" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BG14" t="n">
         <v>0</v>
@@ -3153,17 +3183,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>E. Diouf</t>
+          <t>K. Diatta</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 25</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3173,12 +3203,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>18ibccymsaxom7wdnfz0tevx0</t>
+          <t>f5j3vhj805xtkos7l538u0d7t</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -3195,22 +3225,22 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="S15" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
@@ -3234,25 +3264,25 @@
         <v>0</v>
       </c>
       <c r="AE15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="AG15" t="n">
         <v>1</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>E. Diouf</t>
+          <t>K. Diatta</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>-0.0112303</v>
+        <v>0.1002249899999999</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.45</t>
+          <t>-0.32</t>
         </is>
       </c>
       <c r="AK15" t="n">
@@ -3262,7 +3292,7 @@
         <v>0</v>
       </c>
       <c r="AM15" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3271,22 +3301,22 @@
         <v>0</v>
       </c>
       <c r="AP15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR15" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AS15" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AT15" t="n">
         <v>1</v>
       </c>
       <c r="AU15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AV15" t="n">
         <v>0</v>
@@ -3317,7 +3347,7 @@
         <v>0</v>
       </c>
       <c r="BF15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG15" t="n">
         <v>0</v>
@@ -3336,17 +3366,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>P. Gueye</t>
+          <t>E. Diouf</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 26</t>
+          <t xml:space="preserve"> 25</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3356,12 +3386,12 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ekm47qd8w1x0456lm1tmf5re1</t>
+          <t>18ibccymsaxom7wdnfz0tevx0</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3378,22 +3408,22 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="S16" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
@@ -3417,35 +3447,35 @@
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF16" t="n">
-        <v>-0.05</v>
+        <v>-0.4</v>
       </c>
       <c r="AG16" t="n">
         <v>1</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>P. Gueye</t>
+          <t>E. Diouf</t>
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.2516935299999999</v>
+        <v>-0.10471682</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>-0.18</t>
+          <t>-0.53</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="AL16" t="n">
         <v>0</v>
       </c>
       <c r="AM16" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3454,22 +3484,22 @@
         <v>0</v>
       </c>
       <c r="AP16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ16" t="n">
         <v>0</v>
       </c>
       <c r="AR16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AS16" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AT16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AU16" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV16" t="n">
         <v>0</v>
@@ -3500,7 +3530,7 @@
         <v>0</v>
       </c>
       <c r="BF16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG16" t="n">
         <v>0</v>
@@ -3519,17 +3549,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>K. Koulibaly</t>
+          <t>P. Gueye</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 3</t>
+          <t xml:space="preserve"> 26</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -3539,18 +3569,20 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>b1srdmp4cmwl9k768h8a2ixn9</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr"/>
+          <t>ekm47qd8w1x0456lm1tmf5re1</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>2</v>
+      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -3561,22 +3593,22 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="T17" t="inlineStr"/>
       <c r="U17" t="inlineStr"/>
@@ -3600,35 +3632,35 @@
         <v>0</v>
       </c>
       <c r="AE17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF17" t="n">
-        <v>-0.2</v>
+        <v>-0.1</v>
       </c>
       <c r="AG17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH17" t="inlineStr">
         <is>
-          <t>K. Koulibaly</t>
+          <t>P. Gueye</t>
         </is>
       </c>
       <c r="AI17" t="n">
-        <v>0.32044278</v>
+        <v>0.21994994</v>
       </c>
       <c r="AJ17" t="inlineStr">
         <is>
-          <t>-0.12</t>
+          <t>-0.20</t>
         </is>
       </c>
       <c r="AK17" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="AL17" t="n">
         <v>0</v>
       </c>
       <c r="AM17" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3643,16 +3675,16 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AS17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AT17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV17" t="n">
         <v>0</v>
@@ -3702,17 +3734,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>M. Niakhaté</t>
+          <t>K. Koulibaly</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 19</t>
+          <t xml:space="preserve"> 3</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3722,12 +3754,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>9rf5uk6c2wce30b9wkmu3iuad</t>
+          <t>b1srdmp4cmwl9k768h8a2ixn9</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -3744,22 +3776,22 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3783,35 +3815,35 @@
         <v>0</v>
       </c>
       <c r="AE18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF18" t="n">
-        <v>-0.2</v>
+        <v>-0.4</v>
       </c>
       <c r="AG18" t="n">
         <v>1</v>
       </c>
       <c r="AH18" t="inlineStr">
         <is>
-          <t>M. Niakhaté</t>
+          <t>K. Koulibaly</t>
         </is>
       </c>
       <c r="AI18" t="n">
-        <v>-0.19025539</v>
+        <v>0.14579233</v>
       </c>
       <c r="AJ18" t="inlineStr">
         <is>
-          <t>-0.63</t>
+          <t>-0.27</t>
         </is>
       </c>
       <c r="AK18" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3829,16 +3861,16 @@
         <v>1</v>
       </c>
       <c r="AS18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="AT18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU18" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AW18" t="n">
         <v>0</v>
@@ -3885,17 +3917,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>I. Sarr</t>
+          <t>M. Niakhaté</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 18</t>
+          <t xml:space="preserve"> 19</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3905,12 +3937,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>44s112hd02w1i2ucvai9jy7e1</t>
+          <t>9rf5uk6c2wce30b9wkmu3iuad</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -3927,22 +3959,22 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -3966,35 +3998,35 @@
         <v>0</v>
       </c>
       <c r="AE19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF19" t="n">
-        <v>0</v>
+        <v>-0.4</v>
       </c>
       <c r="AG19" t="n">
         <v>1</v>
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>I. Sarr</t>
+          <t>M. Niakhaté</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>0.5015356</v>
+        <v>-0.36513143</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>+0.07</t>
+          <t>-0.79</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
@@ -4003,16 +4035,16 @@
         <v>0</v>
       </c>
       <c r="AP19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ19" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AR19" t="n">
         <v>1</v>
       </c>
       <c r="AS19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AT19" t="n">
         <v>0</v>
@@ -4021,7 +4053,7 @@
         <v>0</v>
       </c>
       <c r="AV19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW19" t="n">
         <v>0</v>
@@ -4049,7 +4081,7 @@
         <v>0</v>
       </c>
       <c r="BF19" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="BG19" t="n">
         <v>0</v>
@@ -4068,17 +4100,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>I. Gueye</t>
+          <t>I. Sarr</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 5</t>
+          <t xml:space="preserve"> 18</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4088,18 +4120,20 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ceerfv28fygp7m2euv5n5uu39</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr"/>
+          <t>44s112hd02w1i2ucvai9jy7e1</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>2</v>
+      </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -4110,22 +4144,22 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4152,32 +4186,32 @@
         <v>1</v>
       </c>
       <c r="AF20" t="n">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="AG20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>I. Gueye</t>
+          <t>I. Sarr</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>0.14946032</v>
+        <v>0.5048969000000001</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>-0.29</t>
+          <t>+0.08</t>
         </is>
       </c>
       <c r="AK20" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="AL20" t="n">
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4186,13 +4220,13 @@
         <v>0</v>
       </c>
       <c r="AP20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AR20" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="AS20" t="n">
         <v>0</v>
@@ -4201,7 +4235,7 @@
         <v>0</v>
       </c>
       <c r="AU20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV20" t="n">
         <v>0</v>
@@ -4232,7 +4266,7 @@
         <v>0</v>
       </c>
       <c r="BF20" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BG20" t="n">
         <v>0</v>
@@ -4251,17 +4285,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>N. Jackson</t>
+          <t>I. Gueye</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 11</t>
+          <t xml:space="preserve"> 5</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4271,12 +4305,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>amcwh6w0brmkttg4uc5qm6z9w</t>
+          <t>ceerfv28fygp7m2euv5n5uu39</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -4293,22 +4327,22 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -4332,35 +4366,35 @@
         <v>0</v>
       </c>
       <c r="AE21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF21" t="n">
-        <v>0</v>
+        <v>-0.1</v>
       </c>
       <c r="AG21" t="n">
         <v>1</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>N. Jackson</t>
+          <t>I. Gueye</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>0.5975043</v>
+        <v>0.14210678</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>+0.16</t>
+          <t>-0.28</t>
         </is>
       </c>
       <c r="AK21" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="AL21" t="n">
         <v>0</v>
       </c>
       <c r="AM21" t="n">
-        <v>73</v>
+        <v>83</v>
       </c>
       <c r="AN21" t="n">
         <v>0</v>
@@ -4369,22 +4403,22 @@
         <v>0</v>
       </c>
       <c r="AP21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AQ21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR21" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AS21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT21" t="n">
         <v>0</v>
       </c>
       <c r="AU21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV21" t="n">
         <v>0</v>
@@ -4415,7 +4449,7 @@
         <v>0</v>
       </c>
       <c r="BF21" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="BG21" t="n">
         <v>0</v>
@@ -4434,17 +4468,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>L. Camara</t>
+          <t>N. Jackson</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 8</t>
+          <t xml:space="preserve"> 11</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4454,18 +4488,20 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>8eq4c5cotvem9ae9uzb2yezo4</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr"/>
+          <t>amcwh6w0brmkttg4uc5qm6z9w</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>2</v>
+      </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
@@ -4476,22 +4512,22 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>AM</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4515,35 +4551,35 @@
         <v>0</v>
       </c>
       <c r="AE22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AF22" t="n">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="AG22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>L. Camara</t>
+          <t>N. Jackson</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>-0.07019398999999998</v>
+        <v>0.67550506</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>-0.51</t>
+          <t>+0.26</t>
         </is>
       </c>
       <c r="AK22" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="AL22" t="n">
         <v>0</v>
       </c>
       <c r="AM22" t="n">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="AN22" t="n">
         <v>0</v>
@@ -4552,22 +4588,22 @@
         <v>0</v>
       </c>
       <c r="AP22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AQ22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AS22" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AT22" t="n">
         <v>0</v>
       </c>
       <c r="AU22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV22" t="n">
         <v>0</v>
@@ -4598,7 +4634,7 @@
         <v>0</v>
       </c>
       <c r="BF22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BG22" t="n">
         <v>0</v>
@@ -4617,17 +4653,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>S. Mané</t>
+          <t>L. Camara</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10</t>
+          <t xml:space="preserve"> 8</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4637,18 +4673,20 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>cotiiu6mjkfx5xa63nhfbdf4l</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr"/>
+          <t>8eq4c5cotvem9ae9uzb2yezo4</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -4659,22 +4697,22 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>AM</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -4701,32 +4739,32 @@
         <v>1</v>
       </c>
       <c r="AF23" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>S. Mané</t>
+          <t>L. Camara</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>0.20547744</v>
+        <v>-0.07019398999999998</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>-0.23</t>
+          <t>-0.49</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>
@@ -4738,16 +4776,16 @@
         <v>0</v>
       </c>
       <c r="AQ23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR23" t="n">
         <v>3</v>
       </c>
-      <c r="AR23" t="n">
-        <v>2</v>
-      </c>
       <c r="AS23" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AT23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU23" t="n">
         <v>0</v>
@@ -4756,7 +4794,7 @@
         <v>0</v>
       </c>
       <c r="AW23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX23" t="n">
         <v>0</v>
@@ -4781,9 +4819,940 @@
         <v>0</v>
       </c>
       <c r="BF23" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>cqsflhc7vaul90l2d4ipzzzmc</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>S. Mané</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 10</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>cotiiu6mjkfx5xa63nhfbdf4l</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>83</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>83</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="S24" t="n">
+        <v>83</v>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
+      <c r="X24" t="inlineStr"/>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AF24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AH24" t="inlineStr">
+        <is>
+          <t>S. Mané</t>
+        </is>
+      </c>
+      <c r="AI24" t="n">
+        <v>0.23848455</v>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>-0.18</t>
+        </is>
+      </c>
+      <c r="AK24" t="n">
+        <v>13</v>
+      </c>
+      <c r="AL24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM24" t="n">
+        <v>83</v>
+      </c>
+      <c r="AN24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>3</v>
+      </c>
+      <c r="AS24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT24" t="n">
+        <v>2</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF24" t="n">
         <v>4</v>
       </c>
-      <c r="BG23" t="n">
+      <c r="BG24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cqsflhc7vaul90l2d4ipzzzmc</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>B. Dieng</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 9</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>8vlfwoquq3v68mb9ax1pk5fkk</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>82</v>
+      </c>
+      <c r="L25" t="n">
+        <v>2</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>1</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="n">
+        <v>82</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>83</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="S25" t="n">
+        <v>1</v>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
+      <c r="X25" t="inlineStr"/>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr"/>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG25" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH25" t="inlineStr">
+        <is>
+          <t>B. Dieng</t>
+        </is>
+      </c>
+      <c r="AI25" t="n">
+        <v>-0.004268819999999998</v>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>-0.42</t>
+        </is>
+      </c>
+      <c r="AK25" t="n">
+        <v>20</v>
+      </c>
+      <c r="AL25" t="n">
+        <v>82</v>
+      </c>
+      <c r="AM25" t="n">
+        <v>83</v>
+      </c>
+      <c r="AN25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF25" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>cqsflhc7vaul90l2d4ipzzzmc</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>I. Ndiaye</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 13</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>3dm2bfuoyips4rbj0vhvbp9be</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>82</v>
+      </c>
+      <c r="L26" t="n">
+        <v>2</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>1</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="n">
+        <v>82</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>83</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="S26" t="n">
+        <v>1</v>
+      </c>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="inlineStr"/>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr"/>
+      <c r="Y26" t="inlineStr"/>
+      <c r="Z26" t="inlineStr"/>
+      <c r="AA26" t="inlineStr"/>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF26" t="n">
+        <v>-0</v>
+      </c>
+      <c r="AG26" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH26" t="inlineStr">
+        <is>
+          <t>I. Ndiaye</t>
+        </is>
+      </c>
+      <c r="AI26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>-0.42</t>
+        </is>
+      </c>
+      <c r="AK26" t="n">
+        <v>19</v>
+      </c>
+      <c r="AL26" t="n">
+        <v>82</v>
+      </c>
+      <c r="AM26" t="n">
+        <v>83</v>
+      </c>
+      <c r="AN26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF26" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>cqsflhc7vaul90l2d4ipzzzmc</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>I. Mbaye</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 20</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>20eqyvyrgtafzssdh0zaehdsk</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>74</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>9</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="n">
+        <v>74</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>83</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="S27" t="n">
+        <v>9</v>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="inlineStr"/>
+      <c r="W27" t="inlineStr"/>
+      <c r="X27" t="inlineStr"/>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG27" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH27" t="inlineStr">
+        <is>
+          <t>I. Mbaye</t>
+        </is>
+      </c>
+      <c r="AI27" t="n">
+        <v>-0.006432500000000001</v>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>-0.43</t>
+        </is>
+      </c>
+      <c r="AK27" t="n">
+        <v>21</v>
+      </c>
+      <c r="AL27" t="n">
+        <v>74</v>
+      </c>
+      <c r="AM27" t="n">
+        <v>83</v>
+      </c>
+      <c r="AN27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR27" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD27" t="inlineStr"/>
+      <c r="BE27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF27" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cqsflhc7vaul90l2d4ipzzzmc</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>H. Diarra</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 21</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>egtyl4noukbjkm1va1i11e87o</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>75</v>
+      </c>
+      <c r="L28" t="n">
+        <v>2</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>8</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="n">
+        <v>75</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>83</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>AM</t>
+        </is>
+      </c>
+      <c r="S28" t="n">
+        <v>8</v>
+      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+      <c r="X28" t="inlineStr"/>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>2wk1549tkz80oet8226euj7jp</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="AD28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE28" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF28" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="AG28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH28" t="inlineStr">
+        <is>
+          <t>H. Diarra</t>
+        </is>
+      </c>
+      <c r="AI28" t="n">
+        <v>-0.04947731</v>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>-0.47</t>
+        </is>
+      </c>
+      <c r="AK28" t="n">
+        <v>22</v>
+      </c>
+      <c r="AL28" t="n">
+        <v>75</v>
+      </c>
+      <c r="AM28" t="n">
+        <v>83</v>
+      </c>
+      <c r="AN28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR28" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD28" t="inlineStr"/>
+      <c r="BE28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF28" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG28" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>